<commit_message>
Update on script stabilization for R1 and R2
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/LoginData.xlsx
+++ b/src/test/resources/TEST_DATA/LoginData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="18"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="LoginDataAlternateSix" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="LoginDataAlternateSeven" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="LoginDataAlternateEight" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="LoginDataAlternateNine" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>userName</t>
   </si>
@@ -94,51 +95,51 @@
     <t>incorrectPassword</t>
   </si>
   <si>
+    <t>lkp156</t>
+  </si>
+  <si>
+    <t>tgeffrf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS</t>
+  </si>
+  <si>
+    <t>popupText</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are you sure you want to logout?</t>
+  </si>
+  <si>
+    <t>mohanw</t>
+  </si>
+  <si>
+    <t>newPassword</t>
+  </si>
+  <si>
+    <t>Hoax@2345</t>
+  </si>
+  <si>
+    <t>primaryAccountSentSuccessMsg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary Account Set Successful</t>
+  </si>
+  <si>
+    <t>LoginErrorMessage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS: 4</t>
+  </si>
+  <si>
+    <t>shirania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMS sent successfully to the registered mobile number:******9261</t>
+  </si>
+  <si>
     <t>ceftissue</t>
   </si>
   <si>
-    <t>Abcd@1234</t>
-  </si>
-  <si>
-    <t>tgeffrf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS</t>
-  </si>
-  <si>
-    <t>popupText</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Are you sure you want to logout?</t>
-  </si>
-  <si>
-    <t>mohanw</t>
-  </si>
-  <si>
-    <t>newPassword</t>
-  </si>
-  <si>
-    <t>Hoax@2345</t>
-  </si>
-  <si>
-    <t>primaryAccountSentSuccessMsg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primary Account Set Successful</t>
-  </si>
-  <si>
-    <t>LoginErrorMessage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOGIN FAILED! PLEASE RECHECK THE USERNAME AND PASSWORD AND TRY AGAIN. REMAINING LOGIN ATTEMPTS: 4</t>
-  </si>
-  <si>
-    <t>shirania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMS sent successfully to the registered mobile number:******9261</t>
-  </si>
-  <si>
     <t>thishya</t>
   </si>
   <si>
@@ -146,6 +147,9 @@
   </si>
   <si>
     <t>usp2k2</t>
+  </si>
+  <si>
+    <t>safras77</t>
   </si>
 </sst>
 </file>
@@ -188,10 +192,10 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -753,7 +757,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" ht="14.25">
@@ -767,7 +771,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -798,7 +802,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -828,69 +832,69 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="29.421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="29.421875"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="15.57421875"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>29</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="15.57421875"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -898,16 +902,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>7</v>
@@ -944,7 +948,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -979,13 +983,13 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1017,13 +1021,13 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1038,9 +1042,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="9.140625"/>
-    <col customWidth="1" min="2" max="2" style="3" width="13.8515625"/>
-    <col min="3" max="16384" style="3" width="9.140625"/>
+    <col min="1" max="1" style="4" width="9.140625"/>
+    <col customWidth="1" min="2" max="2" style="4" width="13.8515625"/>
+    <col min="3" max="16384" style="4" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1077,9 +1081,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="9.140625"/>
-    <col customWidth="1" min="2" max="2" style="3" width="14.8515625"/>
-    <col min="3" max="16384" style="3" width="9.140625"/>
+    <col min="1" max="1" style="4" width="9.140625"/>
+    <col customWidth="1" min="2" max="2" style="4" width="14.8515625"/>
+    <col min="3" max="16384" style="4" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1095,9 +1099,9 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -1155,7 +1159,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="16384" style="3" width="9.140625"/>
+    <col min="1" max="16384" style="4" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1188,6 +1192,40 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -1230,7 +1268,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.140625"/>
+    <col customWidth="1" min="1" max="1" width="24.8515625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1425,14 +1463,14 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Multiple Payees Click Paynow
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/LoginData.xlsx
+++ b/src/test/resources/TEST_DATA/LoginData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sampath_QA\Automation\svr4-api-automations\svr4-api-automations\src\test\resources\TEST_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E66717B0-DAA9-4326-A217-0B553D748D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6586BDE1-A51F-43CE-9CEF-E7A80241B5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1394,10 +1394,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
Multiple Payees Select option
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/LoginData.xlsx
+++ b/src/test/resources/TEST_DATA/LoginData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sampath_QA\Automation\svr4-api-automations\svr4-api-automations\src\test\resources\TEST_DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6586BDE1-A51F-43CE-9CEF-E7A80241B5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5241F31B-26D5-473C-8A6A-88227EC7B6BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1830" yWindow="-14370" windowWidth="21600" windowHeight="11235" firstSheet="26" activeTab="28" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="68">
   <si>
     <t>userName</t>
   </si>
@@ -249,9 +249,6 @@
   </si>
   <si>
     <t>chan400</t>
-  </si>
-  <si>
-    <t>channad</t>
   </si>
   <si>
     <t>Email sent successfully to the registered email address:</t>
@@ -1357,13 +1354,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>67</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>